<commit_message>
feat(kiddovax): Family-level RFID architecture redesign, child journey assistant, smart queueing, and excel exporter [2026-08-14]
</commit_message>
<xml_diff>
--- a/hospital_credentials.xlsx
+++ b/hospital_credentials.xlsx
@@ -7,7 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Vaccinations" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Hospitals" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Receptionists" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Patients" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Admins" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,143 +417,333 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Hospital Name</t>
+          <t>Vaccine ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Phone Number</t>
+          <t>Vaccine Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Password</t>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Stock Quantity</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Minimum Quantity</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Hospital Title</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Hospital ID</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Jamnabai General Hospital</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2652517401</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2652517401</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MMR</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>500</v>
+      </c>
+      <c r="D2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CityCare Hospital</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>G.M.E.R.S. Hospital Gotri</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2652398000</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2652398000</t>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Hospital ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Hospital Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Contact (Username)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Password</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Doctor Name</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Area</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ESIC Hospital</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2652580360</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2652580360</t>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CityCare Hospital</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>123 Main St</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>TestCity</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>TestArea</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>National Health mission - Aayushman Bharat Government hospital</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1800114477</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1800114477</t>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Receptionist ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Contact (Username)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Password</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Hospital Title</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Hospital ID</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date of Joining</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Shrimati Maniben Thakorbhai Patel Arogya Bhavan</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2652428880</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2652428880</t>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Patient ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Contact (Username)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Password</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Area</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Sanjeevani Aarogya Mandir</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2652750950</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2652750950</t>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Aarav Patel</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>9876543210</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>456 Park Ave</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>TestCity</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>TestArea</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>SSG</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2652424848</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2652424848</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Shree Vallabh Hospital</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>9173781384</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>9173781384</t>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Admin ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Username</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Password</t>
         </is>
       </c>
     </row>

</xml_diff>